<commit_message>
Implement 2-stage Gemini pipeline with confidence scoring and waterfall routing, remove Groq
</commit_message>
<xml_diff>
--- a/Systemdaten/Globale_KontenRegeln.xlsx
+++ b/Systemdaten/Globale_KontenRegeln.xlsx
@@ -7178,7 +7178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1204"/>
+  <dimension ref="A1:G1230"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -13306,7 +13306,6 @@
           <t>HOLZNER METZGEREI - ANDREAS-HOFER-STRASSE 15 - 39011 LANA</t>
         </is>
       </c>
-      <c r="F1030" t="inlineStr"/>
       <c r="G1030" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -15337,7 +15336,6 @@
           <t>HOLZNER GMBH - ANDREAS HOFER STR. 15 - 39011 LANA BZ</t>
         </is>
       </c>
-      <c r="F1085" t="inlineStr"/>
       <c r="G1085" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -15777,7 +15775,6 @@
           <t>LIEFERUNGSNR. 05-25SV13288 VOM 02/12/25</t>
         </is>
       </c>
-      <c r="F1097" t="inlineStr"/>
       <c r="G1097" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -15810,7 +15807,6 @@
           <t>IHRE AUFTRAGSREF. 51002 VOM 01/12/25</t>
         </is>
       </c>
-      <c r="F1098" t="inlineStr"/>
       <c r="G1098" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -15991,7 +15987,6 @@
           <t>LIEFERUNGSNR. 05-25SV13332 VOM 03/12/25</t>
         </is>
       </c>
-      <c r="F1103" t="inlineStr"/>
       <c r="G1103" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16024,7 +16019,6 @@
           <t>IHRE AUFTRAGSREF. 51093 VOM 02/12/25</t>
         </is>
       </c>
-      <c r="F1104" t="inlineStr"/>
       <c r="G1104" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16057,7 +16051,6 @@
           <t>LIEFERUNGSNR. 05-25SV13377 VOM 04/12/25</t>
         </is>
       </c>
-      <c r="F1105" t="inlineStr"/>
       <c r="G1105" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16090,7 +16083,6 @@
           <t>IHRE AUFTRAGSREF. 51209 VOM 03/12/25</t>
         </is>
       </c>
-      <c r="F1106" t="inlineStr"/>
       <c r="G1106" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16197,7 +16189,6 @@
           <t>LIEFERUNGSNR. 05-25SV13421 VOM 05/12/25</t>
         </is>
       </c>
-      <c r="F1109" t="inlineStr"/>
       <c r="G1109" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16230,7 +16221,6 @@
           <t>IHRE AUFTRAGSREF. 51273 VOM 04/12/25</t>
         </is>
       </c>
-      <c r="F1110" t="inlineStr"/>
       <c r="G1110" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16263,7 +16253,6 @@
           <t>LIEFERUNGSNR. 05-25SV13473 VOM 06/12/25</t>
         </is>
       </c>
-      <c r="F1111" t="inlineStr"/>
       <c r="G1111" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16296,7 +16285,6 @@
           <t>IHRE AUFTRAGSREF. 51449 VOM 05/12/25</t>
         </is>
       </c>
-      <c r="F1112" t="inlineStr"/>
       <c r="G1112" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16329,7 +16317,6 @@
           <t>LIEFERUNGSNR. 05-25SV13561 VOM 10/12/25</t>
         </is>
       </c>
-      <c r="F1113" t="inlineStr"/>
       <c r="G1113" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16362,7 +16349,6 @@
           <t>IHRE AUFTRAGSREF. 51654 VOM 09/12/25</t>
         </is>
       </c>
-      <c r="F1114" t="inlineStr"/>
       <c r="G1114" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16395,7 +16381,6 @@
           <t>LIEFERUNGSNR. 05-25SV13653 VOM 12/12/25</t>
         </is>
       </c>
-      <c r="F1115" t="inlineStr"/>
       <c r="G1115" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16428,7 +16413,6 @@
           <t>IHRE AUFTRAGSREF. 51833 VOM 11/12/25</t>
         </is>
       </c>
-      <c r="F1116" t="inlineStr"/>
       <c r="G1116" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16498,7 +16482,6 @@
           <t>LIEFERUNGSNR. 05-25SV13691 VOM 13/12/25</t>
         </is>
       </c>
-      <c r="F1118" t="inlineStr"/>
       <c r="G1118" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -16531,7 +16514,6 @@
           <t>IHRE AUFTRAGSREF. 52016 VOM 12/12/25</t>
         </is>
       </c>
-      <c r="F1119" t="inlineStr"/>
       <c r="G1119" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
@@ -19678,6 +19660,968 @@
         </is>
       </c>
       <c r="G1204" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>02578060218</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>Purnamh GmbH/SRL Società Benefit</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1205" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH HOLZNER ALEXANDER</t>
+        </is>
+      </c>
+      <c r="E1205" t="inlineStr">
+        <is>
+          <t>BERGAPFELSAFT NATUR 0</t>
+        </is>
+      </c>
+      <c r="F1205" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1205" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>00137840203</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>LEVONI S.P.A. Societa Benefit</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1206" t="inlineStr">
+        <is>
+          <t>HOLZNER SRL_.</t>
+        </is>
+      </c>
+      <c r="E1206" t="inlineStr">
+        <is>
+          <t>SALAME UNGHERESE 3</t>
+        </is>
+      </c>
+      <c r="F1206" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1206" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1207" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1207" t="inlineStr">
+        <is>
+          <t>VENTRICINA 2</t>
+        </is>
+      </c>
+      <c r="F1207" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1207" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1208" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1208" t="inlineStr">
+        <is>
+          <t>RIGA AGGIUNTIVA PER SCONTO CUMULATIVO RIGA 1 IN PERCENTUALE 24</t>
+        </is>
+      </c>
+      <c r="F1208" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1208" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1209" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1209" t="inlineStr">
+        <is>
+          <t>GUANCIALE RUSTICO 1</t>
+        </is>
+      </c>
+      <c r="F1209" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1209" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1210" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1210" t="inlineStr">
+        <is>
+          <t>PECORINO DI ROCCA 2</t>
+        </is>
+      </c>
+      <c r="F1210" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1210" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1211" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1211" t="inlineStr">
+        <is>
+          <t>PARMA S/O 18M SPEC 7</t>
+        </is>
+      </c>
+      <c r="F1211" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1211" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1212" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1212" t="inlineStr">
+        <is>
+          <t>SALAME ILGENTILE 1</t>
+        </is>
+      </c>
+      <c r="F1212" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1212" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1213" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1213" t="inlineStr">
+        <is>
+          <t>RIGA AGGIUNTIVA PER SCONTO CUMULATIVO RIGA 6 IN PERCENTUALE 15</t>
+        </is>
+      </c>
+      <c r="F1213" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1213" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1214" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1214" t="inlineStr">
+        <is>
+          <t>FINOCCHIONA IGP 2</t>
+        </is>
+      </c>
+      <c r="F1214" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1214" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1215" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1215" t="inlineStr">
+        <is>
+          <t>RIGA AGGIUNTIVA PER SCONTO CUMULATIVO RIGA 8 IN PERCENTUALE 21</t>
+        </is>
+      </c>
+      <c r="F1215" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1215" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1216" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1216" t="inlineStr">
+        <is>
+          <t>SAL. STOFELOTTO 2</t>
+        </is>
+      </c>
+      <c r="F1216" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1216" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1217" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1217" t="inlineStr">
+        <is>
+          <t>RIGA AGGIUNTIVA PER SCONTO CUMULATIVO RIGA 10 IN PERCENTUALE 19</t>
+        </is>
+      </c>
+      <c r="F1217" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1217" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1218" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1218" t="inlineStr">
+        <is>
+          <t>S. BOCC.FILZE 35G PC1</t>
+        </is>
+      </c>
+      <c r="F1218" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1218" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1219" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1219" t="inlineStr">
+        <is>
+          <t>RIGA AGGIUNTIVA PER SCONTO CUMULATIVO RIGA 12 IN PERCENTUALE 15</t>
+        </is>
+      </c>
+      <c r="F1219" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1219" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1220" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1220" t="inlineStr">
+        <is>
+          <t>CULAT.DIAM S/O SV4</t>
+        </is>
+      </c>
+      <c r="F1220" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1220" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1221" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1221" t="inlineStr">
+        <is>
+          <t>RIGA AGGIUNTIVA PER SCONTO CUMULATIVO RIGA 16 IN PERCENTUALE 4</t>
+        </is>
+      </c>
+      <c r="F1221" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1221" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1222" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1222" t="inlineStr">
+        <is>
+          <t>RIGA AGGIUNTIVA PER SCONTO CUMULATIVO RIGA 18 IN PERCENTUALE 16</t>
+        </is>
+      </c>
+      <c r="F1222" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1222" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>00772580361</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>Villani S.p.A.</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1223" t="inlineStr">
+        <is>
+          <t>HOLZNER GMBH - SRL</t>
+        </is>
+      </c>
+      <c r="E1223" t="inlineStr">
+        <is>
+          <t>RIGA AGGIUNTIVA PER SCONTO CUMULATIVO RIGA 20 IN PERCENTUALE 15</t>
+        </is>
+      </c>
+      <c r="F1223" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1223" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>01192160214</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>Rinner Alexander &amp; CO KG</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1224" t="inlineStr">
+        <is>
+          <t>Holzner GmbH  (Holzner GmbH)</t>
+        </is>
+      </c>
+      <c r="E1224" t="inlineStr">
+        <is>
+          <t>BIO SALAMI PIKANT 1/2</t>
+        </is>
+      </c>
+      <c r="F1224" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1224" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>01192160214</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>Rinner Alexander &amp; CO KG</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1225" t="inlineStr">
+        <is>
+          <t>Holzner GmbH  (Holzner GmbH)</t>
+        </is>
+      </c>
+      <c r="E1225" t="inlineStr">
+        <is>
+          <t>SALAMI MIT REH 1/2</t>
+        </is>
+      </c>
+      <c r="F1225" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1225" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>01192160214</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>Rinner Alexander &amp; CO KG</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1226" t="inlineStr">
+        <is>
+          <t>Holzner GmbH  (Holzner GmbH)</t>
+        </is>
+      </c>
+      <c r="E1226" t="inlineStr">
+        <is>
+          <t>SALAMI MIT HIRSCH 1/2</t>
+        </is>
+      </c>
+      <c r="F1226" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1226" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>01192160214</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>Rinner Alexander &amp; CO KG</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1227" t="inlineStr">
+        <is>
+          <t>Holzner GmbH  (Holzner GmbH)</t>
+        </is>
+      </c>
+      <c r="E1227" t="inlineStr">
+        <is>
+          <t>KRÄUTERSALAMI 1/2</t>
+        </is>
+      </c>
+      <c r="F1227" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1227" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>00101080216</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>Milchhof Meran Gen. u. landw. Ges./Latteria Sociale Merano Soc. Agr. Cop.</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1228" t="inlineStr">
+        <is>
+          <t>Holzner GmbH</t>
+        </is>
+      </c>
+      <c r="E1228" t="inlineStr">
+        <is>
+          <t>FRISCHMILCH 0</t>
+        </is>
+      </c>
+      <c r="F1228" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1228" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>00101080216</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>Milchhof Meran Gen. u. landw. Ges./Latteria Sociale Merano Soc. Agr. Cop.</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1229" t="inlineStr">
+        <is>
+          <t>Holzner GmbH</t>
+        </is>
+      </c>
+      <c r="E1229" t="inlineStr">
+        <is>
+          <t>FRISCHRAHM 0</t>
+        </is>
+      </c>
+      <c r="F1229" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1229" t="inlineStr">
+        <is>
+          <t>AUSSTEHEND</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>01695950210</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>Günther Schmidhammer</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>02977480215</t>
+        </is>
+      </c>
+      <c r="D1230" t="inlineStr">
+        <is>
+          <t>Holzner GmbH</t>
+        </is>
+      </c>
+      <c r="E1230" t="inlineStr">
+        <is>
+          <t>KARTON EIER ZU 180 STÜCK EIER CAT. A GRÖE M/L 0</t>
+        </is>
+      </c>
+      <c r="F1230" t="inlineStr">
+        <is>
+          <t>100 / 801006</t>
+        </is>
+      </c>
+      <c r="G1230" t="inlineStr">
         <is>
           <t>AUSSTEHEND</t>
         </is>

</xml_diff>